<commit_message>
feat: add global chat feature with websocket support
- Added a new chat room page accessible via the '/chat-room' route.
- Implemented websocket connection for real-time messaging in the global chat.
- Created API endpoints for fetching global chat history and online users.
- Updated permissions to include access to the global chat feature.
- Enhanced the database schema to support global chat messages.
- Added UI components for displaying messages, online users, and sending messages.
- Included functionality for image and order card messages in the chat.
</commit_message>
<xml_diff>
--- a/整改与实施计划表2.0.xlsx
+++ b/整改与实施计划表2.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/micropue/Desktop/前后端项目/虎虎校园跑登记系统/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58711073-64E5-D043-BFE4-06E4E86FF98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60545B12-9652-FE45-8E59-EAB3D3E5418E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="1160" windowWidth="27700" windowHeight="16480" xr2:uid="{5E70EDB3-85B7-F849-A4EB-0335214D26D4}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19500" xr2:uid="{5E70EDB3-85B7-F849-A4EB-0335214D26D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>编号</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -138,6 +138,42 @@
   </si>
   <si>
     <t>未支付金额</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>员工内部聊天室</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>支持显示在线状态，上传图片</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1日</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>已支付</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>9月9日前</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>消息列表的起始红点颜色区分</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>已完成</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>9月10</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -272,7 +308,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -291,14 +327,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1">
       <alignment vertical="center"/>
@@ -306,43 +336,16 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="44" fontId="2" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="汇总" xfId="2" builtinId="25"/>
     <cellStyle name="检查单元格" xfId="1" builtinId="23"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -375,21 +378,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -402,11 +390,11 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -430,11 +418,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -861,76 +849,117 @@
       <c r="M2" s="2">
         <v>46251</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="O2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="8" t="s">
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8"/>
+      <c r="S2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="8"/>
-      <c r="U2" s="7"/>
-    </row>
-    <row r="3" spans="1:21" ht="18" thickTop="1" thickBot="1">
+      <c r="T2" s="9"/>
+      <c r="U2" s="6"/>
+    </row>
+    <row r="3" spans="1:21" ht="36" thickTop="1" thickBot="1">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="3">
+        <v>160</v>
+      </c>
+      <c r="F3" s="3">
+        <v>160</v>
+      </c>
       <c r="G3" s="3">
         <f t="shared" ref="G3:G66" si="0">F3-E3</f>
         <v>0</v>
       </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="S3" s="9" t="s">
+      <c r="H3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" s="2">
+        <v>46274</v>
+      </c>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="S3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="9">
+      <c r="T3" s="7">
         <f>SUM(E3:E155)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="18" thickTop="1" thickBot="1">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" ht="36" thickTop="1" thickBot="1">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="C4" s="4"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="D4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
       <c r="G4" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="S4" s="9" t="s">
+      <c r="H4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4" s="2">
+        <v>46274</v>
+      </c>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="S4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="T4" s="9">
+      <c r="T4" s="7">
         <f>SUM(F3:F155)</f>
-        <v>0</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="18" thickTop="1" thickBot="1">
@@ -952,15 +981,15 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="S5" s="9" t="s">
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="S5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="9">
+      <c r="T5" s="7">
         <f>SUMIF(I2:I155,"已支付",F2:F155)</f>
-        <v>0</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="18" thickTop="1" thickBot="1">
@@ -982,13 +1011,13 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="S6" s="9" t="s">
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="S6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="T6" s="9">
+      <c r="T6" s="7">
         <f>T3-T5</f>
         <v>0</v>
       </c>
@@ -1012,9 +1041,9 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
     </row>
     <row r="8" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A8" s="1">
@@ -1035,9 +1064,9 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
     </row>
     <row r="9" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A9" s="1">
@@ -1058,9 +1087,9 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
     </row>
     <row r="10" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A10" s="1">
@@ -1081,9 +1110,9 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
     </row>
     <row r="11" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A11" s="1">
@@ -1104,9 +1133,9 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
     </row>
     <row r="12" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A12" s="1">
@@ -1127,9 +1156,9 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
     </row>
     <row r="13" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A13" s="1">
@@ -1150,9 +1179,9 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
     </row>
     <row r="14" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A14" s="1">
@@ -1173,9 +1202,9 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
     </row>
     <row r="15" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A15" s="1">
@@ -1196,9 +1225,9 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="1:21" ht="18" thickTop="1" thickBot="1">
       <c r="A16" s="1">
@@ -1219,9 +1248,9 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
     </row>
     <row r="17" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A17" s="1">
@@ -1242,9 +1271,9 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
     </row>
     <row r="18" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A18" s="1">
@@ -1265,9 +1294,9 @@
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
     </row>
     <row r="19" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A19" s="1">
@@ -1288,9 +1317,9 @@
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
     </row>
     <row r="20" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A20" s="1">
@@ -1311,9 +1340,9 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="10"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
     </row>
     <row r="21" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A21" s="1">
@@ -1334,9 +1363,9 @@
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
     </row>
     <row r="22" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A22" s="1">
@@ -1357,9 +1386,9 @@
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
     </row>
     <row r="23" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A23" s="1">
@@ -1380,9 +1409,9 @@
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="10"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
     </row>
     <row r="24" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A24" s="1">
@@ -1403,9 +1432,9 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="10"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
     </row>
     <row r="25" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A25" s="1">
@@ -1426,9 +1455,9 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="10"/>
-      <c r="Q25" s="10"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
     </row>
     <row r="26" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A26" s="1">
@@ -1449,9 +1478,9 @@
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="10"/>
-      <c r="Q26" s="10"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
     </row>
     <row r="27" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A27" s="1">
@@ -1472,9 +1501,9 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="10"/>
-      <c r="Q27" s="10"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
     </row>
     <row r="28" spans="1:17" ht="18" thickTop="1" thickBot="1">
       <c r="A28" s="1">
@@ -1495,9 +1524,9 @@
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="10"/>
-      <c r="Q28" s="10"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
     </row>
     <row r="29" spans="1:17" ht="17" thickTop="1">
       <c r="A29" s="1">
@@ -4046,41 +4075,41 @@
     <mergeCell ref="S2:T2"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="D2:D1048576">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"修复"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"新增"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"重构"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:G155">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I155">
+    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
+      <formula>"已支付"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I2:I1048576">
-    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="9" operator="equal">
       <formula>"未支付"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I155">
-    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
-      <formula>"已支付"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J2:J155">
-    <cfRule type="cellIs" dxfId="10" priority="7" operator="equal">
-      <formula>"未完成"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"已完成"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:G155">
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D1048576">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
-      <formula>"重构"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
-      <formula>"新增"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <formula>"修复"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
+      <formula>"未完成"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>